<commit_message>
Promotional Video Shot List
</commit_message>
<xml_diff>
--- a/files/Storyboard_PromoVideo.xlsx
+++ b/files/Storyboard_PromoVideo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peng/西安外国语-人工智能学院/数字人项目/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peng/西安外国语-人工智能学院/数字人项目/XITU-Virtual-Human/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AF082A2-D2FE-8340-A08E-61EA18425703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BD3EFB6-F352-8A4B-898A-235FEC109F87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="960" yWindow="820" windowWidth="28300" windowHeight="17440" xr2:uid="{FEB63B4A-1676-3F42-92B0-4D607159BC06}"/>
+    <workbookView xWindow="120" yWindow="820" windowWidth="28300" windowHeight="17440" xr2:uid="{FEB63B4A-1676-3F42-92B0-4D607159BC06}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
   <si>
     <t xml:space="preserve">镜号
 </t>
@@ -65,6 +65,73 @@
   </si>
   <si>
     <t>备注</t>
+  </si>
+  <si>
+    <t>室内</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>白天</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>空镜起 → 推门进 → 站到数字人前</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>门框作前景框景；地面光带/砖缝为引导线，画面中心留给数字人；</t>
+  </si>
+  <si>
+    <t>Rack Focus：门沿→数字人标记；速度“缓入—匀速—缓出”</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>4-6s</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>无</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主题：</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>吴校长数字人和学生进行多语言的对话</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>数字人拉近景，再推远把学生和数字人放在一个镜头里</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3D数字人</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>数字人放在正中间，展示3d数字人的一些动态</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>30s</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>学生数字人和学生同时出现在画面中间，做打招呼的动作，然后切到数字人上停留1s。最后拉远景，真人（男生）和数字人进行对话</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>男生问数字人：请告诉我旅游学院是个怎样的学院？</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1min</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>女生1（英文）：人工智能时代下外语专业的不可替代性；女生2（法语）：西安外国语大学的学生的职业规划与发展</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -451,10 +518,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C9466E2-9951-1E48-9FCB-E17F213E0AB6}">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="4" max="4" width="36.33203125" customWidth="1"/>
+    <col min="5" max="5" width="25.5" customWidth="1"/>
+    <col min="11" max="11" width="31.5" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="34">
+    <row r="1" spans="1:11" ht="34">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -482,59 +554,135 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="K1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:9">
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4">
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5">
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
-      <c r="A6">
+    <row r="7" spans="1:11">
+      <c r="A7">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7">
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
-      <c r="A8">
+    <row r="9" spans="1:11">
+      <c r="A9">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
-      <c r="A9">
+    <row r="10" spans="1:11">
+      <c r="A10">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
-      <c r="A10">
+    <row r="11" spans="1:11">
+      <c r="A11">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
-      <c r="A11">
+    <row r="12" spans="1:11">
+      <c r="A12">
         <v>10</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>